<commit_message>
[feat] ServiceManager에 NetworkService 이전, 햄스터 외형 변경 기능 구현
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/FaceData.xlsx
+++ b/JsonConverter/ExcelFiles/FaceData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\JagalchiHang\JsonConverter\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\Hamzzi\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B29CAD96-9EC8-4D98-BA93-7E6F2E8D99AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C907C777-0AF5-445C-850F-8F582073D131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시트1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="123">
   <si>
     <r>
       <rPr>
@@ -61,10 +61,6 @@
   </si>
   <si>
     <t>IconPath</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>아이콘 경로</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -389,6 +385,103 @@
   </si>
   <si>
     <t>Hamster/Face_28</t>
+  </si>
+  <si>
+    <t>MaterialPath</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>머테리얼 경로</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>얼굴 아이콘 경로</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_01_Icon</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_02_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_03_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_04_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_05_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_06_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_07_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_08_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_09_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_10_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_11_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_12_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_13_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_14_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_15_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_16_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_17_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_18_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_19_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_20_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_21_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_22_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_23_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_24_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_25_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_26_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_27_Icon</t>
+  </si>
+  <si>
+    <t>Hamster/HamsterIcon/Face_28_Icon</t>
   </si>
 </sst>
 </file>
@@ -709,33 +802,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
     <col min="3" max="3" width="74.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.42578125" customWidth="1"/>
     <col min="7" max="7" width="18.7109375" customWidth="1"/>
     <col min="8" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -745,13 +841,14 @@
       <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="2"/>
+      <c r="E2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -762,397 +859,484 @@
       <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="13.5" x14ac:dyDescent="0.25">
+      <c r="E3" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="13.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D5" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="13.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="6" spans="1:5" ht="13.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="B6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="13.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="7" spans="1:5" ht="13.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D7" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="13.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    <row r="8" spans="1:5" ht="13.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D8" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="13.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+    <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+    <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D10" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+    <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D11" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D12" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D13" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D14" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D15" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+    <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D16" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D17" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+    <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D18" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+    <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D19" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+    <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D20" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D21" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D22" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+    <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D23" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+    <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D24" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+    <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B25" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D25" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+    <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D26" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D27" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+    <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D28" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B29" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D29" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="D31" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>